<commit_message>
Refactor variable naming and update datastructure handling in create_datastructure.py; remove obsolete variable_definition.xlsx and add generated files
</commit_message>
<xml_diff>
--- a/tests/datastructure/example_datastructure.xlsx
+++ b/tests/datastructure/example_datastructure.xlsx
@@ -458,27 +458,27 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>BodemhoogteVak</t>
+          <t>bodemhoogte_vak</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Weerstand_C1_mean</t>
+          <t>c1_mean</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Weerstand_C1_vc</t>
+          <t>c1_vc</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Weerstand_C3_mean</t>
+          <t>c3_mean</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Weerstand_C3_vc</t>
+          <t>c3_vc</t>
         </is>
       </c>
     </row>
@@ -534,22 +534,22 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>DIST_L_GEOM</t>
+          <t>L_intrede</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>DIST_BUT</t>
+          <t>L_but</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>DIST_BIT</t>
+          <t>L_bit</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>DIST_L3</t>
+          <t>L3</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -559,17 +559,17 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>WBN</t>
+          <t>buitenwaterstand</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Bodemhoogte</t>
+          <t>bodemhoogte</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Polderpei</t>
+          <t>polderpeil</t>
         </is>
       </c>
     </row>
@@ -605,42 +605,42 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>ScenarioNaam</t>
+          <t>Scenarionaam</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>ScenarioKans</t>
+          <t>Scenariokans</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Top_zand_mean</t>
+          <t>top_zand_mean</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Top_zand_stdev</t>
+          <t>top_zand_stdev</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>gamma_sat_cover_mean</t>
+          <t>gamma_sat_deklaag_mean</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>gamma_sat_cover_stdev</t>
+          <t>gamma_sat_deklaag_stdev</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>d_wvp_mean</t>
+          <t>D_wvp_mean</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>d_wvp_stdev</t>
+          <t>D_wvp_stdev</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>D70_mean</t>
+          <t>d70_mean</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>D70_vc</t>
+          <t>d70_vc</t>
         </is>
       </c>
     </row>

</xml_diff>